<commit_message>
Update the multi-entity EP sample workbook.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Execution Plan Sample file/MultiEntitySummary.xlsx
+++ b/Execution Plan Sample file/MultiEntitySummary.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -539,9 +539,44 @@
         <v>v1.0</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC-204</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Shared AP rule</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Accounts Payable</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>Life UG, Gen UG</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v>v1.0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>